<commit_message>
feat: nang cap UI solid 100%, bieu do radar ky nang, font Montserrat va ket noi truc tiep Google Sheet
</commit_message>
<xml_diff>
--- a/data/Template_KetQua_HocSinh.xlsx
+++ b/data/Template_KetQua_HocSinh.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:Y21"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -418,9 +418,13 @@
     <col min="16" max="16" width="60.83203125" customWidth="1"/>
     <col min="17" max="17" width="18.83203125" customWidth="1"/>
     <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="60.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
     <col min="20" max="20" width="18.83203125" customWidth="1"/>
     <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="60.83203125" customWidth="1"/>
+    <col min="24" max="24" width="18.83203125" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -473,18 +477,30 @@
         <v>nx_phan_xa</v>
       </c>
       <c r="Q1" t="str">
+        <v>diem_tu_vung</v>
+      </c>
+      <c r="R1" t="str">
+        <v>diem_ngu_phap</v>
+      </c>
+      <c r="S1" t="str">
+        <v>diem_phat_am</v>
+      </c>
+      <c r="T1" t="str">
+        <v>diem_phan_xa</v>
+      </c>
+      <c r="U1" t="str">
         <v>pct_co_ban</v>
       </c>
-      <c r="R1" t="str">
+      <c r="V1" t="str">
         <v>pct_nang_cao</v>
       </c>
-      <c r="S1" t="str">
+      <c r="W1" t="str">
         <v>nhan_xet_lo_trinh</v>
       </c>
-      <c r="T1" t="str">
+      <c r="X1" t="str">
         <v>bac_nang_luc</v>
       </c>
-      <c r="U1" t="str">
+      <c r="Y1" t="str">
         <v>ngay_cap</v>
       </c>
     </row>
@@ -538,18 +554,30 @@
         <v>Con còn rụt rè và có tâm lý sợ sai. Càng về cuối giờ con cởi mở hơn, đã trả lời được cả câu "I'm happy" khi cô hỏi.</v>
       </c>
       <c r="Q2" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="R2" t="str">
+        <v>9.2</v>
+      </c>
+      <c r="S2" t="str">
+        <v>8.6</v>
+      </c>
+      <c r="T2" t="str">
+        <v>9.4</v>
+      </c>
+      <c r="U2" t="str">
         <v>100%</v>
       </c>
-      <c r="R2" t="str">
+      <c r="V2" t="str">
         <v>10%</v>
       </c>
-      <c r="S2" t="str">
+      <c r="W2" t="str">
         <v>Dựa trên kết quả buổi học, trung tâm gợi ý con theo lộ trình cá nhân hoá: củng cố nền tảng phát âm trong 4 buổi đầu, sau đó tăng dần tỷ trọng luyện nói.</v>
       </c>
-      <c r="T2" t="str">
+      <c r="X2" t="str">
         <v>Bậc 1-</v>
       </c>
-      <c r="U2" t="str">
+      <c r="Y2" t="str">
         <v>Hà Nội, ngày 1 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -603,18 +631,30 @@
         <v>Con phản xạ nhanh với câu hỏi quen thuộc, thời gian nghĩ trung bình dưới 3 giây.</v>
       </c>
       <c r="Q3" t="str">
+        <v>8.2</v>
+      </c>
+      <c r="R3" t="str">
+        <v>7.2</v>
+      </c>
+      <c r="S3" t="str">
+        <v>8.0</v>
+      </c>
+      <c r="T3" t="str">
+        <v>7.4</v>
+      </c>
+      <c r="U3" t="str">
         <v>100%</v>
       </c>
-      <c r="R3" t="str">
+      <c r="V3" t="str">
         <v>15%</v>
       </c>
-      <c r="S3" t="str">
+      <c r="W3" t="str">
         <v>Lộ trình đề xuất cho con: 2 buổi/tuần, ưu tiên mở rộng vốn từ theo chủ đề và luyện phản xạ giao tiếp.</v>
       </c>
-      <c r="T3" t="str">
+      <c r="X3" t="str">
         <v>Bậc 1</v>
       </c>
-      <c r="U3" t="str">
+      <c r="Y3" t="str">
         <v>Hà Nội, ngày 2 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -668,18 +708,30 @@
         <v>Con thường trả lời bằng từ đơn. Cô sẽ khuyến khích con mở rộng thành câu đầy đủ bằng cách hỏi thêm "Why?" sau mỗi câu trả lời.</v>
       </c>
       <c r="Q4" t="str">
+        <v>5.8</v>
+      </c>
+      <c r="R4" t="str">
+        <v>6.2</v>
+      </c>
+      <c r="S4" t="str">
+        <v>5.6</v>
+      </c>
+      <c r="T4" t="str">
+        <v>6.4</v>
+      </c>
+      <c r="U4" t="str">
         <v>100%</v>
       </c>
-      <c r="R4" t="str">
+      <c r="V4" t="str">
         <v>20%</v>
       </c>
-      <c r="S4" t="str">
+      <c r="W4" t="str">
         <v>Con phù hợp với lộ trình tăng tốc: học song song kiến thức cơ bản và mở rộng chủ đề nâng cao để chuẩn bị cho các kỳ thi trong năm học.</v>
       </c>
-      <c r="T4" t="str">
+      <c r="X4" t="str">
         <v>Bậc 2</v>
       </c>
-      <c r="U4" t="str">
+      <c r="Y4" t="str">
         <v>Hà Nội, ngày 3 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -733,18 +785,30 @@
         <v>Con chủ động hỏi lại cô khi chưa nghe rõ — đây là thói quen rất tốt cần duy trì.</v>
       </c>
       <c r="Q5" t="str">
+        <v>8.0</v>
+      </c>
+      <c r="R5" t="str">
+        <v>8.4</v>
+      </c>
+      <c r="S5" t="str">
+        <v>7.8</v>
+      </c>
+      <c r="T5" t="str">
+        <v>7.2</v>
+      </c>
+      <c r="U5" t="str">
         <v>100%</v>
       </c>
-      <c r="R5" t="str">
+      <c r="V5" t="str">
         <v>25%</v>
       </c>
-      <c r="S5" t="str">
+      <c r="W5" t="str">
         <v>Trung tâm đề xuất con học nhóm nhỏ 1 kèm 3 để vừa có bạn tương tác, vừa được cô theo sát khi phát âm.</v>
       </c>
-      <c r="T5" t="str">
+      <c r="X5" t="str">
         <v>Bậc 1</v>
       </c>
-      <c r="U5" t="str">
+      <c r="Y5" t="str">
         <v>Hà Nội, ngày 4 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -798,18 +862,30 @@
         <v>Con cần tăng môi trường giao tiếp để bớt phụ thuộc vào việc dịch sang tiếng Việt trong đầu trước khi nói.</v>
       </c>
       <c r="Q6" t="str">
+        <v>8.4</v>
+      </c>
+      <c r="R6" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="S6" t="str">
+        <v>9.6</v>
+      </c>
+      <c r="T6" t="str">
+        <v>9.0</v>
+      </c>
+      <c r="U6" t="str">
         <v>100%</v>
       </c>
-      <c r="R6" t="str">
+      <c r="V6" t="str">
         <v>10%</v>
       </c>
-      <c r="S6" t="str">
+      <c r="W6" t="str">
         <v>Dựa trên kết quả buổi học, trung tâm gợi ý con theo lộ trình cá nhân hoá: củng cố nền tảng phát âm trong 4 buổi đầu, sau đó tăng dần tỷ trọng luyện nói.</v>
       </c>
-      <c r="T6" t="str">
+      <c r="X6" t="str">
         <v>Bậc 3</v>
       </c>
-      <c r="U6" t="str">
+      <c r="Y6" t="str">
         <v>Hà Nội, ngày 5 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -863,18 +939,30 @@
         <v>Con tự tin tương tác, dám nói dù chưa chắc đúng. Cô đánh giá cao tinh thần này.</v>
       </c>
       <c r="Q7" t="str">
+        <v>6.2</v>
+      </c>
+      <c r="R7" t="str">
+        <v>6.6</v>
+      </c>
+      <c r="S7" t="str">
+        <v>6.0</v>
+      </c>
+      <c r="T7" t="str">
+        <v>6.8</v>
+      </c>
+      <c r="U7" t="str">
         <v>100%</v>
       </c>
-      <c r="R7" t="str">
+      <c r="V7" t="str">
         <v>15%</v>
       </c>
-      <c r="S7" t="str">
+      <c r="W7" t="str">
         <v>Lộ trình đề xuất cho con: 2 buổi/tuần, ưu tiên mở rộng vốn từ theo chủ đề và luyện phản xạ giao tiếp.</v>
       </c>
-      <c r="T7" t="str">
+      <c r="X7" t="str">
         <v>Bậc 1-</v>
       </c>
-      <c r="U7" t="str">
+      <c r="Y7" t="str">
         <v>Hà Nội, ngày 6 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -928,18 +1016,30 @@
         <v>Con còn rụt rè và có tâm lý sợ sai. Càng về cuối giờ con cởi mở hơn, đã trả lời được cả câu "I'm happy" khi cô hỏi.</v>
       </c>
       <c r="Q8" t="str">
+        <v>5.4</v>
+      </c>
+      <c r="R8" t="str">
+        <v>4.4</v>
+      </c>
+      <c r="S8" t="str">
+        <v>5.2</v>
+      </c>
+      <c r="T8" t="str">
+        <v>4.6</v>
+      </c>
+      <c r="U8" t="str">
         <v>100%</v>
       </c>
-      <c r="R8" t="str">
+      <c r="V8" t="str">
         <v>20%</v>
       </c>
-      <c r="S8" t="str">
+      <c r="W8" t="str">
         <v>Con phù hợp với lộ trình tăng tốc: học song song kiến thức cơ bản và mở rộng chủ đề nâng cao để chuẩn bị cho các kỳ thi trong năm học.</v>
       </c>
-      <c r="T8" t="str">
+      <c r="X8" t="str">
         <v>Bậc 2</v>
       </c>
-      <c r="U8" t="str">
+      <c r="Y8" t="str">
         <v>Hà Nội, ngày 7 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -993,18 +1093,30 @@
         <v>Con phản xạ nhanh với câu hỏi quen thuộc, thời gian nghĩ trung bình dưới 3 giây.</v>
       </c>
       <c r="Q9" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="R9" t="str">
+        <v>9.2</v>
+      </c>
+      <c r="S9" t="str">
+        <v>8.6</v>
+      </c>
+      <c r="T9" t="str">
+        <v>9.4</v>
+      </c>
+      <c r="U9" t="str">
         <v>100%</v>
       </c>
-      <c r="R9" t="str">
+      <c r="V9" t="str">
         <v>25%</v>
       </c>
-      <c r="S9" t="str">
+      <c r="W9" t="str">
         <v>Trung tâm đề xuất con học nhóm nhỏ 1 kèm 3 để vừa có bạn tương tác, vừa được cô theo sát khi phát âm.</v>
       </c>
-      <c r="T9" t="str">
+      <c r="X9" t="str">
         <v>Bậc 1-</v>
       </c>
-      <c r="U9" t="str">
+      <c r="Y9" t="str">
         <v>Hà Nội, ngày 8 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1058,18 +1170,30 @@
         <v>Con thường trả lời bằng từ đơn. Cô sẽ khuyến khích con mở rộng thành câu đầy đủ bằng cách hỏi thêm "Why?" sau mỗi câu trả lời.</v>
       </c>
       <c r="Q10" t="str">
+        <v>8.2</v>
+      </c>
+      <c r="R10" t="str">
+        <v>7.2</v>
+      </c>
+      <c r="S10" t="str">
+        <v>8.0</v>
+      </c>
+      <c r="T10" t="str">
+        <v>7.4</v>
+      </c>
+      <c r="U10" t="str">
         <v>100%</v>
       </c>
-      <c r="R10" t="str">
+      <c r="V10" t="str">
         <v>10%</v>
       </c>
-      <c r="S10" t="str">
+      <c r="W10" t="str">
         <v>Dựa trên kết quả buổi học, trung tâm gợi ý con theo lộ trình cá nhân hoá: củng cố nền tảng phát âm trong 4 buổi đầu, sau đó tăng dần tỷ trọng luyện nói.</v>
       </c>
-      <c r="T10" t="str">
+      <c r="X10" t="str">
         <v>Bậc 1</v>
       </c>
-      <c r="U10" t="str">
+      <c r="Y10" t="str">
         <v>Hà Nội, ngày 9 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1123,18 +1247,30 @@
         <v>Con chủ động hỏi lại cô khi chưa nghe rõ — đây là thói quen rất tốt cần duy trì.</v>
       </c>
       <c r="Q11" t="str">
+        <v>5.8</v>
+      </c>
+      <c r="R11" t="str">
+        <v>6.2</v>
+      </c>
+      <c r="S11" t="str">
+        <v>5.6</v>
+      </c>
+      <c r="T11" t="str">
+        <v>6.4</v>
+      </c>
+      <c r="U11" t="str">
         <v>100%</v>
       </c>
-      <c r="R11" t="str">
+      <c r="V11" t="str">
         <v>15%</v>
       </c>
-      <c r="S11" t="str">
+      <c r="W11" t="str">
         <v>Lộ trình đề xuất cho con: 2 buổi/tuần, ưu tiên mở rộng vốn từ theo chủ đề và luyện phản xạ giao tiếp.</v>
       </c>
-      <c r="T11" t="str">
+      <c r="X11" t="str">
         <v>Bậc 2</v>
       </c>
-      <c r="U11" t="str">
+      <c r="Y11" t="str">
         <v>Hà Nội, ngày 10 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1188,18 +1324,30 @@
         <v>Con cần tăng môi trường giao tiếp để bớt phụ thuộc vào việc dịch sang tiếng Việt trong đầu trước khi nói.</v>
       </c>
       <c r="Q12" t="str">
+        <v>8.0</v>
+      </c>
+      <c r="R12" t="str">
+        <v>8.4</v>
+      </c>
+      <c r="S12" t="str">
+        <v>7.8</v>
+      </c>
+      <c r="T12" t="str">
+        <v>7.2</v>
+      </c>
+      <c r="U12" t="str">
         <v>100%</v>
       </c>
-      <c r="R12" t="str">
+      <c r="V12" t="str">
         <v>20%</v>
       </c>
-      <c r="S12" t="str">
+      <c r="W12" t="str">
         <v>Con phù hợp với lộ trình tăng tốc: học song song kiến thức cơ bản và mở rộng chủ đề nâng cao để chuẩn bị cho các kỳ thi trong năm học.</v>
       </c>
-      <c r="T12" t="str">
+      <c r="X12" t="str">
         <v>Bậc 1</v>
       </c>
-      <c r="U12" t="str">
+      <c r="Y12" t="str">
         <v>Hà Nội, ngày 11 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1253,18 +1401,30 @@
         <v>Con tự tin tương tác, dám nói dù chưa chắc đúng. Cô đánh giá cao tinh thần này.</v>
       </c>
       <c r="Q13" t="str">
+        <v>8.4</v>
+      </c>
+      <c r="R13" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="S13" t="str">
+        <v>9.6</v>
+      </c>
+      <c r="T13" t="str">
+        <v>9.0</v>
+      </c>
+      <c r="U13" t="str">
         <v>100%</v>
       </c>
-      <c r="R13" t="str">
+      <c r="V13" t="str">
         <v>25%</v>
       </c>
-      <c r="S13" t="str">
+      <c r="W13" t="str">
         <v>Trung tâm đề xuất con học nhóm nhỏ 1 kèm 3 để vừa có bạn tương tác, vừa được cô theo sát khi phát âm.</v>
       </c>
-      <c r="T13" t="str">
+      <c r="X13" t="str">
         <v>Bậc 3</v>
       </c>
-      <c r="U13" t="str">
+      <c r="Y13" t="str">
         <v>Hà Nội, ngày 12 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1318,18 +1478,30 @@
         <v>Con còn rụt rè và có tâm lý sợ sai. Càng về cuối giờ con cởi mở hơn, đã trả lời được cả câu "I'm happy" khi cô hỏi.</v>
       </c>
       <c r="Q14" t="str">
+        <v>6.2</v>
+      </c>
+      <c r="R14" t="str">
+        <v>6.6</v>
+      </c>
+      <c r="S14" t="str">
+        <v>6.0</v>
+      </c>
+      <c r="T14" t="str">
+        <v>6.8</v>
+      </c>
+      <c r="U14" t="str">
         <v>100%</v>
       </c>
-      <c r="R14" t="str">
+      <c r="V14" t="str">
         <v>10%</v>
       </c>
-      <c r="S14" t="str">
+      <c r="W14" t="str">
         <v>Dựa trên kết quả buổi học, trung tâm gợi ý con theo lộ trình cá nhân hoá: củng cố nền tảng phát âm trong 4 buổi đầu, sau đó tăng dần tỷ trọng luyện nói.</v>
       </c>
-      <c r="T14" t="str">
+      <c r="X14" t="str">
         <v>Bậc 1-</v>
       </c>
-      <c r="U14" t="str">
+      <c r="Y14" t="str">
         <v>Hà Nội, ngày 13 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1383,18 +1555,30 @@
         <v>Con phản xạ nhanh với câu hỏi quen thuộc, thời gian nghĩ trung bình dưới 3 giây.</v>
       </c>
       <c r="Q15" t="str">
+        <v>5.4</v>
+      </c>
+      <c r="R15" t="str">
+        <v>4.4</v>
+      </c>
+      <c r="S15" t="str">
+        <v>5.2</v>
+      </c>
+      <c r="T15" t="str">
+        <v>4.6</v>
+      </c>
+      <c r="U15" t="str">
         <v>100%</v>
       </c>
-      <c r="R15" t="str">
+      <c r="V15" t="str">
         <v>15%</v>
       </c>
-      <c r="S15" t="str">
+      <c r="W15" t="str">
         <v>Lộ trình đề xuất cho con: 2 buổi/tuần, ưu tiên mở rộng vốn từ theo chủ đề và luyện phản xạ giao tiếp.</v>
       </c>
-      <c r="T15" t="str">
+      <c r="X15" t="str">
         <v>Bậc 2</v>
       </c>
-      <c r="U15" t="str">
+      <c r="Y15" t="str">
         <v>Hà Nội, ngày 14 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1448,18 +1632,30 @@
         <v>Con thường trả lời bằng từ đơn. Cô sẽ khuyến khích con mở rộng thành câu đầy đủ bằng cách hỏi thêm "Why?" sau mỗi câu trả lời.</v>
       </c>
       <c r="Q16" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="R16" t="str">
+        <v>9.2</v>
+      </c>
+      <c r="S16" t="str">
+        <v>8.6</v>
+      </c>
+      <c r="T16" t="str">
+        <v>9.4</v>
+      </c>
+      <c r="U16" t="str">
         <v>100%</v>
       </c>
-      <c r="R16" t="str">
+      <c r="V16" t="str">
         <v>20%</v>
       </c>
-      <c r="S16" t="str">
+      <c r="W16" t="str">
         <v>Con phù hợp với lộ trình tăng tốc: học song song kiến thức cơ bản và mở rộng chủ đề nâng cao để chuẩn bị cho các kỳ thi trong năm học.</v>
       </c>
-      <c r="T16" t="str">
+      <c r="X16" t="str">
         <v>Bậc 1-</v>
       </c>
-      <c r="U16" t="str">
+      <c r="Y16" t="str">
         <v>Hà Nội, ngày 15 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1513,18 +1709,30 @@
         <v>Con chủ động hỏi lại cô khi chưa nghe rõ — đây là thói quen rất tốt cần duy trì.</v>
       </c>
       <c r="Q17" t="str">
+        <v>8.2</v>
+      </c>
+      <c r="R17" t="str">
+        <v>7.2</v>
+      </c>
+      <c r="S17" t="str">
+        <v>8.0</v>
+      </c>
+      <c r="T17" t="str">
+        <v>7.4</v>
+      </c>
+      <c r="U17" t="str">
         <v>100%</v>
       </c>
-      <c r="R17" t="str">
+      <c r="V17" t="str">
         <v>25%</v>
       </c>
-      <c r="S17" t="str">
+      <c r="W17" t="str">
         <v>Trung tâm đề xuất con học nhóm nhỏ 1 kèm 3 để vừa có bạn tương tác, vừa được cô theo sát khi phát âm.</v>
       </c>
-      <c r="T17" t="str">
+      <c r="X17" t="str">
         <v>Bậc 1</v>
       </c>
-      <c r="U17" t="str">
+      <c r="Y17" t="str">
         <v>Hà Nội, ngày 16 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1578,18 +1786,30 @@
         <v>Con cần tăng môi trường giao tiếp để bớt phụ thuộc vào việc dịch sang tiếng Việt trong đầu trước khi nói.</v>
       </c>
       <c r="Q18" t="str">
+        <v>5.8</v>
+      </c>
+      <c r="R18" t="str">
+        <v>6.2</v>
+      </c>
+      <c r="S18" t="str">
+        <v>5.6</v>
+      </c>
+      <c r="T18" t="str">
+        <v>6.4</v>
+      </c>
+      <c r="U18" t="str">
         <v>100%</v>
       </c>
-      <c r="R18" t="str">
+      <c r="V18" t="str">
         <v>10%</v>
       </c>
-      <c r="S18" t="str">
+      <c r="W18" t="str">
         <v>Dựa trên kết quả buổi học, trung tâm gợi ý con theo lộ trình cá nhân hoá: củng cố nền tảng phát âm trong 4 buổi đầu, sau đó tăng dần tỷ trọng luyện nói.</v>
       </c>
-      <c r="T18" t="str">
+      <c r="X18" t="str">
         <v>Bậc 2</v>
       </c>
-      <c r="U18" t="str">
+      <c r="Y18" t="str">
         <v>Hà Nội, ngày 17 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1643,18 +1863,30 @@
         <v>Con tự tin tương tác, dám nói dù chưa chắc đúng. Cô đánh giá cao tinh thần này.</v>
       </c>
       <c r="Q19" t="str">
+        <v>8.0</v>
+      </c>
+      <c r="R19" t="str">
+        <v>8.4</v>
+      </c>
+      <c r="S19" t="str">
+        <v>7.8</v>
+      </c>
+      <c r="T19" t="str">
+        <v>7.2</v>
+      </c>
+      <c r="U19" t="str">
         <v>100%</v>
       </c>
-      <c r="R19" t="str">
+      <c r="V19" t="str">
         <v>15%</v>
       </c>
-      <c r="S19" t="str">
+      <c r="W19" t="str">
         <v>Lộ trình đề xuất cho con: 2 buổi/tuần, ưu tiên mở rộng vốn từ theo chủ đề và luyện phản xạ giao tiếp.</v>
       </c>
-      <c r="T19" t="str">
+      <c r="X19" t="str">
         <v>Bậc 1</v>
       </c>
-      <c r="U19" t="str">
+      <c r="Y19" t="str">
         <v>Hà Nội, ngày 18 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1708,18 +1940,30 @@
         <v>Con còn rụt rè và có tâm lý sợ sai. Càng về cuối giờ con cởi mở hơn, đã trả lời được cả câu "I'm happy" khi cô hỏi.</v>
       </c>
       <c r="Q20" t="str">
+        <v>8.4</v>
+      </c>
+      <c r="R20" t="str">
+        <v>8.8</v>
+      </c>
+      <c r="S20" t="str">
+        <v>9.6</v>
+      </c>
+      <c r="T20" t="str">
+        <v>9.0</v>
+      </c>
+      <c r="U20" t="str">
         <v>100%</v>
       </c>
-      <c r="R20" t="str">
+      <c r="V20" t="str">
         <v>20%</v>
       </c>
-      <c r="S20" t="str">
+      <c r="W20" t="str">
         <v>Con phù hợp với lộ trình tăng tốc: học song song kiến thức cơ bản và mở rộng chủ đề nâng cao để chuẩn bị cho các kỳ thi trong năm học.</v>
       </c>
-      <c r="T20" t="str">
+      <c r="X20" t="str">
         <v>Bậc 3</v>
       </c>
-      <c r="U20" t="str">
+      <c r="Y20" t="str">
         <v>Hà Nội, ngày 19 tháng 3 năm 2026</v>
       </c>
     </row>
@@ -1773,24 +2017,36 @@
         <v>Con phản xạ nhanh với câu hỏi quen thuộc, thời gian nghĩ trung bình dưới 3 giây.</v>
       </c>
       <c r="Q21" t="str">
+        <v>6.2</v>
+      </c>
+      <c r="R21" t="str">
+        <v>6.6</v>
+      </c>
+      <c r="S21" t="str">
+        <v>6.0</v>
+      </c>
+      <c r="T21" t="str">
+        <v>6.8</v>
+      </c>
+      <c r="U21" t="str">
         <v>100%</v>
       </c>
-      <c r="R21" t="str">
+      <c r="V21" t="str">
         <v>25%</v>
       </c>
-      <c r="S21" t="str">
+      <c r="W21" t="str">
         <v>Trung tâm đề xuất con học nhóm nhỏ 1 kèm 3 để vừa có bạn tương tác, vừa được cô theo sát khi phát âm.</v>
       </c>
-      <c r="T21" t="str">
+      <c r="X21" t="str">
         <v>Bậc 1-</v>
       </c>
-      <c r="U21" t="str">
+      <c r="Y21" t="str">
         <v>Hà Nội, ngày 20 tháng 3 năm 2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>